<commit_message>
Modify the Test Cases to Run on Jenkins
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -1,9 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C809B952-9C5B-4E0A-BFA8-3FD970E07426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace2\OrangeHRMProject\src\test\resources\testdata\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9BB06C6-33EC-46EE-B164-509064728223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,7 +17,6 @@
     <sheet name="inValidLoginData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:N15"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -36,23 +40,26 @@
     <t>admin1</t>
   </si>
   <si>
-    <t>orangehrm_rahul</t>
-  </si>
-  <si>
-    <t>Orangehrm_rahul1</t>
+    <t>Admin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -75,8 +82,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -359,6 +367,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -369,11 +381,11 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>